<commit_message>
restructure code and rebase for kafedra=directory with file2
</commit_message>
<xml_diff>
--- a/Файл 1.xlsx
+++ b/Файл 1.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="153222"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25128"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\sysprofiles.adm.vvsu.ru\emplprofiles$\antonov\Desktop\2026.02\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Qweeck\PycharmProjects\vvsu_project\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C51D89E-7533-4AFB-B8B5-9AFA915F3C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="14655" windowHeight="11265"/>
+    <workbookView xWindow="2895" yWindow="2220" windowWidth="21600" windowHeight="13965" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="file" sheetId="2" r:id="rId1"/>
@@ -17,7 +18,19 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">file!$A$7:$AN$435</definedName>
   </definedNames>
-  <calcPr calcId="152511"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1431,7 +1444,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
@@ -2137,7 +2150,7 @@
     <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2151,24 +2164,21 @@
     <xf numFmtId="0" fontId="21" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="34" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2179,18 +2189,6 @@
     <xf numFmtId="0" fontId="21" fillId="33" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2198,15 +2196,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -2225,6 +2214,27 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2265,7 +2275,7 @@
     <cellStyle name="Название" xfId="1" builtinId="15" customBuiltin="1"/>
     <cellStyle name="Нейтральный" xfId="8" builtinId="28" customBuiltin="1"/>
     <cellStyle name="Обычный" xfId="0" builtinId="0"/>
-    <cellStyle name="Обычный 2" xfId="42"/>
+    <cellStyle name="Обычный 2" xfId="42" xr:uid="{00000000-0005-0000-0000-000024000000}"/>
     <cellStyle name="Плохой" xfId="7" builtinId="27" customBuiltin="1"/>
     <cellStyle name="Пояснение" xfId="16" builtinId="53" customBuiltin="1"/>
     <cellStyle name="Примечание" xfId="15" builtinId="10" customBuiltin="1"/>
@@ -2553,7 +2563,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AR435"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
@@ -2598,20 +2608,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.2">
-      <c r="A1" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="15"/>
-      <c r="C1" s="15"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="15"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="15"/>
-      <c r="H1" s="15"/>
-      <c r="I1" s="15"/>
-      <c r="J1" s="15"/>
-      <c r="K1" s="15"/>
-      <c r="L1" s="15"/>
+      <c r="A1" s="23" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="23"/>
+      <c r="C1" s="23"/>
+      <c r="D1" s="23"/>
+      <c r="E1" s="23"/>
+      <c r="F1" s="23"/>
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
     </row>
     <row r="2" spans="1:44" x14ac:dyDescent="0.2">
       <c r="A2" s="7"/>
@@ -2628,167 +2638,167 @@
       <c r="L2" s="7"/>
     </row>
     <row r="3" spans="1:44" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="C3" s="16" t="s">
+      <c r="C3" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="D3" s="16" t="s">
+      <c r="D3" s="24" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="24" t="s">
         <v>5</v>
       </c>
-      <c r="F3" s="19" t="s">
+      <c r="F3" s="14" t="s">
         <v>6</v>
       </c>
-      <c r="G3" s="20"/>
-      <c r="H3" s="21"/>
-      <c r="I3" s="19" t="s">
+      <c r="G3" s="15"/>
+      <c r="H3" s="16"/>
+      <c r="I3" s="14" t="s">
         <v>7</v>
       </c>
-      <c r="J3" s="20"/>
-      <c r="K3" s="20"/>
-      <c r="L3" s="20"/>
-      <c r="M3" s="20"/>
-      <c r="N3" s="20"/>
-      <c r="O3" s="20"/>
-      <c r="P3" s="20"/>
-      <c r="Q3" s="20"/>
-      <c r="R3" s="20"/>
-      <c r="S3" s="20"/>
-      <c r="T3" s="20"/>
-      <c r="U3" s="20"/>
-      <c r="V3" s="20"/>
-      <c r="W3" s="20"/>
-      <c r="X3" s="21"/>
-      <c r="Y3" s="19" t="s">
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15"/>
+      <c r="T3" s="15"/>
+      <c r="U3" s="15"/>
+      <c r="V3" s="15"/>
+      <c r="W3" s="15"/>
+      <c r="X3" s="16"/>
+      <c r="Y3" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="Z3" s="20"/>
-      <c r="AA3" s="20"/>
-      <c r="AB3" s="20"/>
-      <c r="AC3" s="20"/>
-      <c r="AD3" s="20"/>
-      <c r="AE3" s="20"/>
-      <c r="AF3" s="20"/>
-      <c r="AG3" s="20"/>
-      <c r="AH3" s="20"/>
-      <c r="AI3" s="20"/>
-      <c r="AJ3" s="20"/>
-      <c r="AK3" s="20"/>
-      <c r="AL3" s="20"/>
-      <c r="AM3" s="20"/>
-      <c r="AN3" s="21"/>
+      <c r="Z3" s="15"/>
+      <c r="AA3" s="15"/>
+      <c r="AB3" s="15"/>
+      <c r="AC3" s="15"/>
+      <c r="AD3" s="15"/>
+      <c r="AE3" s="15"/>
+      <c r="AF3" s="15"/>
+      <c r="AG3" s="15"/>
+      <c r="AH3" s="15"/>
+      <c r="AI3" s="15"/>
+      <c r="AJ3" s="15"/>
+      <c r="AK3" s="15"/>
+      <c r="AL3" s="15"/>
+      <c r="AM3" s="15"/>
+      <c r="AN3" s="16"/>
       <c r="AO3" s="5"/>
       <c r="AP3" s="5"/>
     </row>
     <row r="4" spans="1:44" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="17"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="17"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="23"/>
-      <c r="H4" s="24"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="26"/>
-      <c r="K4" s="26"/>
-      <c r="L4" s="26"/>
-      <c r="M4" s="26"/>
-      <c r="N4" s="26"/>
-      <c r="O4" s="26"/>
-      <c r="P4" s="26"/>
-      <c r="Q4" s="26"/>
-      <c r="R4" s="26"/>
-      <c r="S4" s="26"/>
-      <c r="T4" s="26"/>
-      <c r="U4" s="26"/>
-      <c r="V4" s="26"/>
-      <c r="W4" s="26"/>
-      <c r="X4" s="27"/>
-      <c r="Y4" s="25" t="s">
+      <c r="A4" s="25"/>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="27"/>
+      <c r="G4" s="28"/>
+      <c r="H4" s="29"/>
+      <c r="I4" s="27"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
+      <c r="O4" s="18"/>
+      <c r="P4" s="18"/>
+      <c r="Q4" s="18"/>
+      <c r="R4" s="18"/>
+      <c r="S4" s="18"/>
+      <c r="T4" s="18"/>
+      <c r="U4" s="18"/>
+      <c r="V4" s="18"/>
+      <c r="W4" s="18"/>
+      <c r="X4" s="19"/>
+      <c r="Y4" s="17" t="s">
         <v>9</v>
       </c>
-      <c r="Z4" s="26"/>
-      <c r="AA4" s="26"/>
-      <c r="AB4" s="26"/>
-      <c r="AC4" s="26"/>
-      <c r="AD4" s="26"/>
-      <c r="AE4" s="26"/>
-      <c r="AF4" s="26"/>
-      <c r="AG4" s="26"/>
-      <c r="AH4" s="26"/>
-      <c r="AI4" s="26"/>
-      <c r="AJ4" s="26"/>
-      <c r="AK4" s="26"/>
-      <c r="AL4" s="26"/>
-      <c r="AM4" s="26"/>
-      <c r="AN4" s="27"/>
+      <c r="Z4" s="18"/>
+      <c r="AA4" s="18"/>
+      <c r="AB4" s="18"/>
+      <c r="AC4" s="18"/>
+      <c r="AD4" s="18"/>
+      <c r="AE4" s="18"/>
+      <c r="AF4" s="18"/>
+      <c r="AG4" s="18"/>
+      <c r="AH4" s="18"/>
+      <c r="AI4" s="18"/>
+      <c r="AJ4" s="18"/>
+      <c r="AK4" s="18"/>
+      <c r="AL4" s="18"/>
+      <c r="AM4" s="18"/>
+      <c r="AN4" s="19"/>
       <c r="AO4" s="5"/>
       <c r="AP4" s="5"/>
     </row>
     <row r="5" spans="1:44" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A5" s="17"/>
-      <c r="B5" s="17"/>
-      <c r="C5" s="17"/>
-      <c r="D5" s="17"/>
-      <c r="E5" s="17"/>
-      <c r="F5" s="25"/>
-      <c r="G5" s="26"/>
-      <c r="H5" s="27"/>
-      <c r="I5" s="25"/>
-      <c r="J5" s="28"/>
-      <c r="K5" s="28"/>
-      <c r="L5" s="28"/>
-      <c r="M5" s="28"/>
-      <c r="N5" s="28"/>
-      <c r="O5" s="28"/>
-      <c r="P5" s="29"/>
-      <c r="Q5" s="30" t="s">
+      <c r="A5" s="25"/>
+      <c r="B5" s="25"/>
+      <c r="C5" s="25"/>
+      <c r="D5" s="25"/>
+      <c r="E5" s="25"/>
+      <c r="F5" s="17"/>
+      <c r="G5" s="18"/>
+      <c r="H5" s="19"/>
+      <c r="I5" s="17"/>
+      <c r="J5" s="20"/>
+      <c r="K5" s="20"/>
+      <c r="L5" s="20"/>
+      <c r="M5" s="20"/>
+      <c r="N5" s="20"/>
+      <c r="O5" s="20"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="R5" s="28"/>
-      <c r="S5" s="28"/>
-      <c r="T5" s="28"/>
-      <c r="U5" s="28"/>
-      <c r="V5" s="28"/>
-      <c r="W5" s="28"/>
-      <c r="X5" s="29"/>
-      <c r="Y5" s="30" t="s">
+      <c r="R5" s="20"/>
+      <c r="S5" s="20"/>
+      <c r="T5" s="20"/>
+      <c r="U5" s="20"/>
+      <c r="V5" s="20"/>
+      <c r="W5" s="20"/>
+      <c r="X5" s="21"/>
+      <c r="Y5" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="Z5" s="28"/>
-      <c r="AA5" s="28"/>
-      <c r="AB5" s="28"/>
-      <c r="AC5" s="28"/>
-      <c r="AD5" s="28"/>
-      <c r="AE5" s="28"/>
-      <c r="AF5" s="29"/>
-      <c r="AG5" s="30" t="s">
+      <c r="Z5" s="20"/>
+      <c r="AA5" s="20"/>
+      <c r="AB5" s="20"/>
+      <c r="AC5" s="20"/>
+      <c r="AD5" s="20"/>
+      <c r="AE5" s="20"/>
+      <c r="AF5" s="21"/>
+      <c r="AG5" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="AH5" s="28"/>
-      <c r="AI5" s="28"/>
-      <c r="AJ5" s="28"/>
-      <c r="AK5" s="28"/>
-      <c r="AL5" s="28"/>
-      <c r="AM5" s="28"/>
-      <c r="AN5" s="29"/>
+      <c r="AH5" s="20"/>
+      <c r="AI5" s="20"/>
+      <c r="AJ5" s="20"/>
+      <c r="AK5" s="20"/>
+      <c r="AL5" s="20"/>
+      <c r="AM5" s="20"/>
+      <c r="AN5" s="21"/>
       <c r="AO5" s="5"/>
       <c r="AP5" s="5"/>
     </row>
     <row r="6" spans="1:44" ht="14.25" x14ac:dyDescent="0.2">
-      <c r="A6" s="18"/>
-      <c r="B6" s="18"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="18"/>
-      <c r="E6" s="18"/>
+      <c r="A6" s="26"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
       <c r="F6" s="2" t="s">
         <v>12</v>
       </c>
@@ -2900,10 +2910,10 @@
       <c r="AP6" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="AQ6" s="11" t="s">
+      <c r="AQ6" s="5" t="s">
         <v>465</v>
       </c>
-      <c r="AR6" s="11" t="s">
+      <c r="AR6" s="5" t="s">
         <v>467</v>
       </c>
     </row>
@@ -16297,7 +16307,7 @@
       <c r="J105" s="4">
         <v>92.5</v>
       </c>
-      <c r="K105" s="14">
+      <c r="K105" s="13">
         <v>618</v>
       </c>
       <c r="L105" s="4">
@@ -22697,7 +22707,7 @@
       <c r="J153" s="4">
         <v>67</v>
       </c>
-      <c r="K153" s="14">
+      <c r="K153" s="13">
         <v>420</v>
       </c>
       <c r="L153" s="4">
@@ -26147,7 +26157,7 @@
       <c r="J178" s="4">
         <v>300.26</v>
       </c>
-      <c r="K178" s="12">
+      <c r="K178" s="11">
         <v>442</v>
       </c>
       <c r="L178" s="4">
@@ -55843,7 +55853,7 @@
       <c r="J394" s="4">
         <v>42.5</v>
       </c>
-      <c r="K394" s="13">
+      <c r="K394" s="12">
         <v>1262.5</v>
       </c>
       <c r="L394" s="4">
@@ -58741,7 +58751,7 @@
       <c r="J415" s="4">
         <v>92</v>
       </c>
-      <c r="K415" s="12">
+      <c r="K415" s="11">
         <v>705</v>
       </c>
       <c r="L415" s="4">
@@ -61476,14 +61486,8 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A7:AN435"/>
+  <autoFilter ref="A7:AN435" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <mergeCells count="16">
-    <mergeCell ref="Y3:AN3"/>
-    <mergeCell ref="Y4:AN4"/>
-    <mergeCell ref="J5:P5"/>
-    <mergeCell ref="Q5:X5"/>
-    <mergeCell ref="Y5:AF5"/>
-    <mergeCell ref="AG5:AN5"/>
     <mergeCell ref="A1:L1"/>
     <mergeCell ref="A3:A6"/>
     <mergeCell ref="B3:B6"/>
@@ -61494,6 +61498,12 @@
     <mergeCell ref="I3:I5"/>
     <mergeCell ref="J3:X3"/>
     <mergeCell ref="J4:X4"/>
+    <mergeCell ref="Y3:AN3"/>
+    <mergeCell ref="Y4:AN4"/>
+    <mergeCell ref="J5:P5"/>
+    <mergeCell ref="Q5:X5"/>
+    <mergeCell ref="Y5:AF5"/>
+    <mergeCell ref="AG5:AN5"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>